<commit_message>
Actualizar datos de planes de justicia (2026-07-30)
</commit_message>
<xml_diff>
--- a/data/plan_justicia/cubos_completos_plan_justicia.xlsx
+++ b/data/plan_justicia/cubos_completos_plan_justicia.xlsx
@@ -4635,7 +4635,7 @@
         <v>11849</v>
       </c>
       <c r="G159">
-        <v>2367</v>
+        <v>2376</v>
       </c>
       <c r="H159">
         <v>2935</v>
@@ -14905,7 +14905,7 @@
         <v>742</v>
       </c>
       <c r="G554">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H554">
         <v>75</v>
@@ -43661,7 +43661,7 @@
         <v>9120</v>
       </c>
       <c r="G1660">
-        <v>795</v>
+        <v>815</v>
       </c>
       <c r="H1660">
         <v>1966</v>
@@ -49823,7 +49823,7 @@
         <v>5317</v>
       </c>
       <c r="G1897">
-        <v>745</v>
+        <v>750</v>
       </c>
       <c r="H1897">
         <v>914</v>

</xml_diff>